<commit_message>
added the goal plan.
</commit_message>
<xml_diff>
--- a/C. Financeiro.xlsx
+++ b/C. Financeiro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rcssi\Code\Personal_Finance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FF3BD6B-CC85-4E6A-9921-31AE8957C48A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BECF5E8A-ACE0-4A34-BE3A-98D39D10FE81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-114" yWindow="-114" windowWidth="19704" windowHeight="11178" tabRatio="797" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,8 +18,12 @@
     <sheet name="Receita Líquida" sheetId="8" state="hidden" r:id="rId3"/>
     <sheet name="Despesas Gerais" sheetId="1" state="hidden" r:id="rId4"/>
     <sheet name="Gráfico Categorias" sheetId="14" state="hidden" r:id="rId5"/>
-    <sheet name="Gráfico Anual" sheetId="13" r:id="rId6"/>
+    <sheet name="Objetivos" sheetId="16" state="hidden" r:id="rId6"/>
+    <sheet name="Gráfico Anual" sheetId="13" r:id="rId7"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId8"/>
+  </externalReferences>
   <definedNames>
     <definedName name="Contas">'Validação de Dados'!$B$5:$B$8</definedName>
     <definedName name="Dash">'Gráfico Anual'!$A$1:$P$26</definedName>
@@ -75,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="88">
   <si>
     <t>Mês</t>
   </si>
@@ -321,6 +325,24 @@
   </si>
   <si>
     <t>Conta</t>
+  </si>
+  <si>
+    <t>Iphone</t>
+  </si>
+  <si>
+    <t>Console PS5</t>
+  </si>
+  <si>
+    <t>*Faça alterações nos objetivos e em seus valores como preferir.</t>
+  </si>
+  <si>
+    <t>Objetivo</t>
+  </si>
+  <si>
+    <t>Progresso</t>
+  </si>
+  <si>
+    <t>Viagem</t>
   </si>
 </sst>
 </file>
@@ -615,7 +637,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="44" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -809,6 +831,13 @@
     <xf numFmtId="44" fontId="4" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -9173,6 +9202,40 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Data Validation"/>
+      <sheetName val="Balance &amp; Tracking"/>
+      <sheetName val="Net Salary"/>
+      <sheetName val="Expenses"/>
+      <sheetName val="Graphic Categories"/>
+      <sheetName val="Goals"/>
+      <sheetName val="Graphic Annual"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1">
+        <row r="12">
+          <cell r="C12">
+            <v>0</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{739BA625-5E32-4F47-8323-C47308DEF24A}" name="Tabela1" displayName="Tabela1" ref="B16:H20" insertRowShift="1" totalsRowShown="0" headerRowDxfId="9">
   <autoFilter ref="B16:H20" xr:uid="{739BA625-5E32-4F47-8323-C47308DEF24A}"/>
@@ -15321,6 +15384,233 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E64D7343-0B79-46A5-8FCF-1D91A6E6BF30}">
+  <dimension ref="C2:I16"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="3.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" style="1" customWidth="1"/>
+    <col min="4" max="6" width="17.140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="1"/>
+    <col min="8" max="9" width="14.28515625" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C2" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="3:9" ht="15" x14ac:dyDescent="0.3">
+      <c r="D4" s="44" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="44" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="44" t="s">
+        <v>86</v>
+      </c>
+      <c r="H4" s="44" t="s">
+        <v>81</v>
+      </c>
+      <c r="I4" s="44" t="str">
+        <f>'Saldo &amp; Mov.'!B12</f>
+        <v>Poupança</v>
+      </c>
+    </row>
+    <row r="5" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D5" s="74" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" s="85">
+        <v>4000</v>
+      </c>
+      <c r="F5" s="83">
+        <f t="shared" ref="F5:F16" ca="1" si="0">$I$5/E5</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="84" t="s">
+        <v>2</v>
+      </c>
+      <c r="I5" s="85">
+        <f ca="1">'[1]Balance &amp; Tracking'!C12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D6" s="74" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" s="85">
+        <v>4500</v>
+      </c>
+      <c r="F6" s="83">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D7" s="74" t="s">
+        <v>60</v>
+      </c>
+      <c r="E7" s="85">
+        <v>30000</v>
+      </c>
+      <c r="F7" s="83">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D8" s="74" t="s">
+        <v>87</v>
+      </c>
+      <c r="E8" s="85">
+        <v>5000</v>
+      </c>
+      <c r="F8" s="83">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D9" s="74" t="s">
+        <v>85</v>
+      </c>
+      <c r="E9" s="85">
+        <v>1</v>
+      </c>
+      <c r="F9" s="83">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D10" s="74" t="s">
+        <v>85</v>
+      </c>
+      <c r="E10" s="85">
+        <v>1</v>
+      </c>
+      <c r="F10" s="83">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D11" s="74" t="s">
+        <v>85</v>
+      </c>
+      <c r="E11" s="85">
+        <v>1</v>
+      </c>
+      <c r="F11" s="83">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D12" s="74" t="s">
+        <v>85</v>
+      </c>
+      <c r="E12" s="85">
+        <v>1</v>
+      </c>
+      <c r="F12" s="83">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D13" s="74" t="s">
+        <v>85</v>
+      </c>
+      <c r="E13" s="85">
+        <v>1</v>
+      </c>
+      <c r="F13" s="83">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D14" s="74" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14" s="85">
+        <v>1</v>
+      </c>
+      <c r="F14" s="83">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D15" s="74" t="s">
+        <v>85</v>
+      </c>
+      <c r="E15" s="85">
+        <v>1</v>
+      </c>
+      <c r="F15" s="83">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D16" s="74" t="s">
+        <v>85</v>
+      </c>
+      <c r="E16" s="85">
+        <v>1</v>
+      </c>
+      <c r="F16" s="83">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="F5:F16">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{05B70BAD-B629-4120-AE30-6272C3F126ED}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{05B70BAD-B629-4120-AE30-6272C3F126ED}">
+            <x14:dataBar minLength="0" maxLength="100">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>1</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>F5:F16</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAD330F4-3FAE-447F-BF05-82EFBCBD7BD0}">
   <sheetPr codeName="Planilha6">
     <tabColor theme="1"/>
@@ -15373,15 +15663,15 @@
         <v>41</v>
       </c>
       <c r="J2" s="3"/>
-      <c r="K2" s="83" t="s">
+      <c r="K2" s="86" t="s">
         <v>24</v>
       </c>
-      <c r="L2" s="84"/>
+      <c r="L2" s="87"/>
       <c r="M2" s="37"/>
-      <c r="N2" s="83" t="s">
+      <c r="N2" s="86" t="s">
         <v>7</v>
       </c>
-      <c r="O2" s="84"/>
+      <c r="O2" s="87"/>
       <c r="P2" s="38"/>
     </row>
     <row r="3" spans="1:16" ht="15" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
fixing terminology for bank account, and adjusting zoom.
</commit_message>
<xml_diff>
--- a/C. Financeiro.xlsx
+++ b/C. Financeiro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rcssi\Code\Personal_Finance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C269ED6-8162-483B-8B49-9C9F06CD655F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FF3BD6B-CC85-4E6A-9921-31AE8957C48A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-114" yWindow="-114" windowWidth="19704" windowHeight="11178" tabRatio="797" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
     <sheet name="Gráfico Anual" sheetId="13" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="Ativos">'Validação de Dados'!$B$5:$B$7</definedName>
+    <definedName name="Contas">'Validação de Dados'!$B$5:$B$8</definedName>
     <definedName name="Dash">'Gráfico Anual'!$A$1:$P$26</definedName>
     <definedName name="Despesas">'Validação de Dados'!$D$5:$D$16</definedName>
     <definedName name="Investimentos">'Validação de Dados'!$F$5:$F$6</definedName>
@@ -29,7 +29,7 @@
     <definedName name="Perdas">'Validação de Dados'!$H$5:$H$9</definedName>
     <definedName name="Receita_Líquida">'Validação de Dados'!$N$5:$N$16</definedName>
     <definedName name="Receitas">'Validação de Dados'!$J$5:$J$9</definedName>
-    <definedName name="Transferir">'Validação de Dados'!$L$5:$L$7</definedName>
+    <definedName name="Transferir">'Validação de Dados'!$L$5:$L$8</definedName>
     <definedName name="Z_12641207_4FA9_4498_AEA1_9BC1962A4F9A_.wvu.Rows" localSheetId="3" hidden="1">'Despesas Gerais'!$6:$6,'Despesas Gerais'!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -191,9 +191,6 @@
     <t>Inss</t>
   </si>
   <si>
-    <t>Alocação</t>
-  </si>
-  <si>
     <t>Operação</t>
   </si>
   <si>
@@ -207,9 +204,6 @@
   </si>
   <si>
     <t>Sld. Anual</t>
-  </si>
-  <si>
-    <t>Sld. Real</t>
   </si>
   <si>
     <t>Diferença</t>
@@ -275,9 +269,6 @@
     <t>Desp./ Receitas</t>
   </si>
   <si>
-    <t>Ativos</t>
-  </si>
-  <si>
     <t>Meses</t>
   </si>
   <si>
@@ -321,6 +312,15 @@
   </si>
   <si>
     <t>*Faça alterações nos valores em azul como preferir, porém para adicionar ou remover valores será necessário alterar a planilha onde for preciso.</t>
+  </si>
+  <si>
+    <t>Contas</t>
+  </si>
+  <si>
+    <t>Poupança</t>
+  </si>
+  <si>
+    <t>Conta</t>
   </si>
 </sst>
 </file>
@@ -9186,7 +9186,7 @@
     </tableColumn>
     <tableColumn id="6" xr3:uid="{23818CCC-08C7-4066-9B86-98D831460C75}" name="Operação" dataDxfId="6"/>
     <tableColumn id="3" xr3:uid="{78815540-1C3C-4370-A3E4-1C8E033CFC39}" name="Categoria" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{F153B94E-6C60-4C63-A86C-8519A94E1F13}" name="Alocação" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{F153B94E-6C60-4C63-A86C-8519A94E1F13}" name="Conta" dataDxfId="4"/>
     <tableColumn id="4" xr3:uid="{EE54C9A2-2D53-4D6A-93DF-88B691A8C3D9}" name="Valor" dataDxfId="3" dataCellStyle="Moeda"/>
     <tableColumn id="5" xr3:uid="{28149A80-D409-4A63-B4C2-6EDA92C21F54}" name="Descrição" dataDxfId="2"/>
   </tableColumns>
@@ -9508,12 +9508,12 @@
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="2:16" ht="15" x14ac:dyDescent="0.3">
       <c r="B4" s="44" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="D4" s="44" t="s">
         <v>1</v>
@@ -9522,19 +9522,19 @@
         <v>3</v>
       </c>
       <c r="H4" s="44" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="J4" s="44" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L4" s="44" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="N4" s="44" t="s">
         <v>16</v>
       </c>
       <c r="P4" s="44" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.25">
@@ -9545,7 +9545,7 @@
         <v>21</v>
       </c>
       <c r="F5" s="74" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H5" s="74" t="s">
         <v>37</v>
@@ -9554,7 +9554,7 @@
         <v>26</v>
       </c>
       <c r="L5" s="75" t="str" cm="1">
-        <f t="array" ref="L5:L7">Ativos</f>
+        <f t="array" ref="L5:L8">Contas</f>
         <v>Banco 1</v>
       </c>
       <c r="N5" s="75" t="str" cm="1">
@@ -9562,7 +9562,7 @@
         <v>Salário</v>
       </c>
       <c r="P5" s="75" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.25">
@@ -9570,13 +9570,13 @@
         <v>31</v>
       </c>
       <c r="D6" s="74" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F6" s="74" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H6" s="74" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="J6" s="74" t="s">
         <v>36</v>
@@ -9588,7 +9588,7 @@
         <v>Vendas</v>
       </c>
       <c r="P6" s="75" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.25">
@@ -9596,13 +9596,13 @@
         <v>27</v>
       </c>
       <c r="D7" s="74" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H7" s="74" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J7" s="74" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="L7" s="75" t="str">
         <v>Carteira</v>
@@ -9611,41 +9611,47 @@
         <v>Aluguel</v>
       </c>
       <c r="P7" s="75" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B8" s="74" t="s">
+        <v>80</v>
+      </c>
       <c r="D8" s="74" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H8" s="74" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J8" s="74" t="s">
-        <v>49</v>
+        <v>47</v>
+      </c>
+      <c r="L8" s="75" t="str">
+        <v>Poupança</v>
       </c>
       <c r="N8" s="75" t="str">
         <v>Rendimentos</v>
       </c>
       <c r="P8" s="75" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D9" s="74" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="H9" s="74" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J9" s="74" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N9" s="75" t="str">
         <v>Receitas Outros</v>
       </c>
       <c r="P9" s="75" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="2:16" x14ac:dyDescent="0.25">
@@ -9657,51 +9663,51 @@
         <v>Inss</v>
       </c>
       <c r="P10" s="75" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D11" s="74" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="N11" s="75" t="str">
         <v>T. Transporte</v>
       </c>
       <c r="P11" s="75" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D12" s="74" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="N12" s="75" t="str">
         <v>Taxa</v>
       </c>
       <c r="P12" s="75" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D13" s="74" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="N13" s="75" t="str">
         <v>Imposto de Renda</v>
       </c>
       <c r="P13" s="75" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D14" s="74" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N14" s="75" t="str">
         <v>Perdas Outros</v>
       </c>
       <c r="P14" s="75" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.25">
@@ -9713,7 +9719,7 @@
         <v>CDI</v>
       </c>
       <c r="P15" s="75" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="2:16" x14ac:dyDescent="0.25">
@@ -9724,7 +9730,7 @@
         <v>Tesouro Direto</v>
       </c>
       <c r="P16" s="75" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -9755,13 +9761,13 @@
     <row r="1" spans="1:8" ht="3.6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:8" ht="14.3" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="44" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C2" s="44" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="72" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F2" s="70" t="s">
         <v>25</v>
@@ -9787,7 +9793,7 @@
     </row>
     <row r="4" spans="1:8" ht="14.3" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="57" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C4" s="73">
         <f>HLOOKUP(B2,'Despesas Gerais'!B2:M20,19,FALSE)/HLOOKUP(B2,'Receita Líquida'!B2:M16,15,FALSE)</f>
@@ -9819,7 +9825,7 @@
     </row>
     <row r="6" spans="1:8" ht="14.3" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="27" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C6" s="26">
         <f>'Gráfico Anual'!I15</f>
@@ -9844,7 +9850,7 @@
     </row>
     <row r="8" spans="1:8" ht="14.3" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="44" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C8" s="44" t="s">
         <v>2</v>
@@ -9859,11 +9865,11 @@
     </row>
     <row r="9" spans="1:8" ht="14.3" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="27" t="str" cm="1">
-        <f t="array" ref="B9:B11">Ativos</f>
+        <f t="array" ref="B9:B12">Contas</f>
         <v>Banco 1</v>
       </c>
       <c r="C9" s="2" cm="1">
-        <f t="array" aca="1" ref="C9" ca="1">SUM(SUMIFS(Tabela1[Valor],Tabela1[Operação],{"Receitas";"Transferir"},Tabela1[Alocação],B9,Tabela1[Data],"&lt;="&amp;(TODAY())))-SUMIFS(Tabela1[Valor],Tabela1[Operação],"&lt;&gt;Receitas",Tabela1[Operação],"&lt;&gt;Transferir",Tabela1[Alocação],B9,Tabela1[Data],"&lt;="&amp;(TODAY())) - SUMIFS(Tabela1[Valor],Tabela1[Categoria],B9,Tabela1[Data],"&lt;="&amp;(TODAY()))</f>
+        <f t="array" aca="1" ref="C9" ca="1">SUM(SUMIFS(Tabela1[Valor],Tabela1[Operação],{"Receitas";"Transferir"},Tabela1[Conta],B9,Tabela1[Data],"&lt;="&amp;(TODAY())))-SUMIFS(Tabela1[Valor],Tabela1[Operação],"&lt;&gt;Receitas",Tabela1[Operação],"&lt;&gt;Transferir",Tabela1[Conta],B9,Tabela1[Data],"&lt;="&amp;(TODAY())) - SUMIFS(Tabela1[Valor],Tabela1[Categoria],B9,Tabela1[Data],"&lt;="&amp;(TODAY()))</f>
         <v>150</v>
       </c>
       <c r="E9" s="69" t="str">
@@ -9880,7 +9886,7 @@
         <v>Banco 2</v>
       </c>
       <c r="C10" s="2" cm="1">
-        <f t="array" aca="1" ref="C10" ca="1">SUM(SUMIFS(Tabela1[Valor],Tabela1[Operação],{"Receitas";"Transferir"},Tabela1[Alocação],B10,Tabela1[Data],"&lt;="&amp;(TODAY())))-SUMIFS(Tabela1[Valor],Tabela1[Operação],"&lt;&gt;Receitas",Tabela1[Operação],"&lt;&gt;Transferir",Tabela1[Alocação],B10,Tabela1[Data],"&lt;="&amp;(TODAY())) - SUMIFS(Tabela1[Valor],Tabela1[Categoria],B10,Tabela1[Data],"&lt;="&amp;(TODAY()))</f>
+        <f t="array" aca="1" ref="C10" ca="1">SUM(SUMIFS(Tabela1[Valor],Tabela1[Operação],{"Receitas";"Transferir"},Tabela1[Conta],B10,Tabela1[Data],"&lt;="&amp;(TODAY())))-SUMIFS(Tabela1[Valor],Tabela1[Operação],"&lt;&gt;Receitas",Tabela1[Operação],"&lt;&gt;Transferir",Tabela1[Conta],B10,Tabela1[Data],"&lt;="&amp;(TODAY())) - SUMIFS(Tabela1[Valor],Tabela1[Categoria],B10,Tabela1[Data],"&lt;="&amp;(TODAY()))</f>
         <v>0</v>
       </c>
       <c r="E10" s="69" t="str">
@@ -9897,7 +9903,7 @@
         <v>Carteira</v>
       </c>
       <c r="C11" s="2" cm="1">
-        <f t="array" aca="1" ref="C11" ca="1">SUM(SUMIFS(Tabela1[Valor],Tabela1[Operação],{"Receitas";"Transferir"},Tabela1[Alocação],B11,Tabela1[Data],"&lt;="&amp;(TODAY())))-SUMIFS(Tabela1[Valor],Tabela1[Operação],"&lt;&gt;Receitas",Tabela1[Operação],"&lt;&gt;Transferir",Tabela1[Alocação],B11,Tabela1[Data],"&lt;="&amp;(TODAY())) - SUMIFS(Tabela1[Valor],Tabela1[Categoria],B11,Tabela1[Data],"&lt;="&amp;(TODAY()))</f>
+        <f t="array" aca="1" ref="C11" ca="1">SUM(SUMIFS(Tabela1[Valor],Tabela1[Operação],{"Receitas";"Transferir"},Tabela1[Conta],B11,Tabela1[Data],"&lt;="&amp;(TODAY())))-SUMIFS(Tabela1[Valor],Tabela1[Operação],"&lt;&gt;Receitas",Tabela1[Operação],"&lt;&gt;Transferir",Tabela1[Conta],B11,Tabela1[Data],"&lt;="&amp;(TODAY())) - SUMIFS(Tabela1[Valor],Tabela1[Categoria],B11,Tabela1[Data],"&lt;="&amp;(TODAY()))</f>
         <v>0</v>
       </c>
       <c r="E11" s="69" t="str">
@@ -9910,12 +9916,12 @@
     </row>
     <row r="12" spans="1:8" ht="14.3" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="59"/>
-      <c r="B12" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="2">
-        <f ca="1">SUM(C9:C11)</f>
-        <v>150</v>
+      <c r="B12" s="27" t="str">
+        <v>Poupança</v>
+      </c>
+      <c r="C12" s="2" cm="1">
+        <f t="array" aca="1" ref="C12" ca="1">SUM(SUMIFS(Tabela1[Valor],Tabela1[Operação],{"Receitas";"Transferir"},Tabela1[Conta],B12,Tabela1[Data],"&lt;="&amp;(TODAY())))-SUMIFS(Tabela1[Valor],Tabela1[Operação],"&lt;&gt;Receitas",Tabela1[Operação],"&lt;&gt;Transferir",Tabela1[Conta],B12,Tabela1[Data],"&lt;="&amp;(TODAY())) - SUMIFS(Tabela1[Valor],Tabela1[Categoria],B12,Tabela1[Data],"&lt;="&amp;(TODAY()))</f>
+        <v>0</v>
       </c>
       <c r="E12" s="69" t="str">
         <v>Rolê/ Entret.</v>
@@ -9928,10 +9934,10 @@
     <row r="13" spans="1:8" ht="14.3" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="59"/>
       <c r="B13" s="27" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C13" s="26">
-        <f ca="1">ROUND(C5-C12,2)</f>
+        <f ca="1">ROUND(C5-SUM(C9:C12),2)</f>
         <v>0</v>
       </c>
       <c r="E13" s="69" t="str">
@@ -9969,13 +9975,13 @@
         <v>0</v>
       </c>
       <c r="D16" s="29" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E16" s="30" t="s">
         <v>33</v>
       </c>
       <c r="F16" s="30" t="s">
-        <v>38</v>
+        <v>81</v>
       </c>
       <c r="G16" s="31" t="s">
         <v>25</v>
@@ -9993,7 +9999,7 @@
         <v>Janeiro</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E17" s="34" t="s">
         <v>26</v>
@@ -13275,7 +13281,7 @@
       <formula1>"Receitas, Perdas, Investimentos, Despesas, Transferir"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F17:F257" xr:uid="{0D51CC9B-6F94-4F85-BAFC-26C786BB30BC}">
-      <formula1>Ativos</formula1>
+      <formula1>Contas</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{D9270E47-B020-4CBF-A3A9-E523B28C14E7}">
       <formula1>Meses</formula1>
@@ -15086,7 +15092,7 @@
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B2" s="44" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C2" s="44" t="s">
         <v>26</v>
@@ -15364,7 +15370,7 @@
         <v>17</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J2" s="3"/>
       <c r="K2" s="83" t="s">

</xml_diff>